<commit_message>
Adicao da remocao de dias nao comerciais
</commit_message>
<xml_diff>
--- a/resumo.xlsx
+++ b/resumo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,105 +441,428 @@
       <c r="E1" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="F1" s="1" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>24/04/2024</t>
-        </is>
+      <c r="A2" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>01/04/2024</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Crédito à vista</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>199.48</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>290.26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>309.16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>365.86</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>534.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01/04/2024</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>579.41</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>15/04/2024</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>653.8099999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08/04/2024</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>15/04/2024</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>747.41</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15/04/2024</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>22/04/2024</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>757.3099999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15/04/2024</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>22/04/2024</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>825.8099999999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>22/04/2024</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>29/04/2024</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>238.83</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>25/04/2024</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Visa</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Crédito à vista</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>30/04/2024</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>780.3100000000001</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>27/04/2024</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Visa</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Crédito à vista</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>02/05/2024</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>924.1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>28/04/2024</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Visa</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Crédito à vista</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>03/05/2024</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>1413.28</v>
+      <c r="F13" t="n">
+        <v>925.01</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>29/04/2024</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>06/05/2024</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>957.1799999999999</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>29/04/2024</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>06/05/2024</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1023.22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>29/04/2024</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Crédito à vista</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>06/05/2024</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1099.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>